<commit_message>
updated site glossary for 1.5.8
</commit_message>
<xml_diff>
--- a/data_files/Site glossary.xlsx
+++ b/data_files/Site glossary.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nih.sharepoint.com/sites/NCI-CBIIT-FNLCCDI/Shared Documents/CCDC (Data Catalog nee PODCat)/2-Executing/System Document/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="188" documentId="13_ncr:1_{CD305CA4-F6E6-494C-8D70-07316997D1EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B74640D5-A2E0-4A20-9BF4-23D0A9324AD6}"/>
+  <xr:revisionPtr revIDLastSave="206" documentId="13_ncr:1_{CD305CA4-F6E6-494C-8D70-07316997D1EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{90C75E1B-174C-4937-9867-F59B97C3FF63}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{4110CF64-F05A-4DD9-960E-BC3FCD1C46EE}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{4110CF64-F05A-4DD9-960E-BC3FCD1C46EE}"/>
   </bookViews>
   <sheets>
     <sheet name="Site glossary" sheetId="2" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="420" uniqueCount="289">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="435" uniqueCount="299">
   <si>
     <t>Term Category</t>
   </si>
@@ -185,9 +185,6 @@
     <t>CIViC</t>
   </si>
   <si>
-    <t>Clinical Interpretations of Variants in Cancer</t>
-  </si>
-  <si>
     <t>CLIA</t>
   </si>
   <si>
@@ -905,14 +902,47 @@
     <t>NF-OSI</t>
   </si>
   <si>
-    <t>NF Data Portal</t>
+    <t>caDSR</t>
+  </si>
+  <si>
+    <t>Cancer Data Standards Registry and Repository</t>
+  </si>
+  <si>
+    <t>FrESCO</t>
+  </si>
+  <si>
+    <t>Framework for Exploring Scalable Computational Oncology</t>
+  </si>
+  <si>
+    <t>PMTL</t>
+  </si>
+  <si>
+    <t>Pediatric Molecular Target Lists</t>
+  </si>
+  <si>
+    <t>STQ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Spatial Transcriptomics Quantification </t>
+  </si>
+  <si>
+    <t>Batch-processing Abstraction for Raw Data Integration</t>
+  </si>
+  <si>
+    <t>BARDI</t>
+  </si>
+  <si>
+    <t>Clinical Interpretation of Variants in Cancer</t>
+  </si>
+  <si>
+    <t>Neurofibromatosis Data Portal Open Science Initiative</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -960,6 +990,13 @@
       <family val="2"/>
       <charset val="1"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -969,7 +1006,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -1005,12 +1042,27 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF4472C4"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF4472C4"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1042,6 +1094,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1357,7 +1410,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{69208F35-5666-473F-97EF-CB7A96B85984}">
-  <dimension ref="A1:E130"/>
+  <dimension ref="A1:E135"/>
   <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="36.453125" bestFit="1" customWidth="1"/>
@@ -1581,7 +1634,7 @@
         <v>47</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>48</v>
+        <v>297</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.35">
@@ -1589,27 +1642,27 @@
         <v>20</v>
       </c>
       <c r="B18" t="s">
+        <v>48</v>
+      </c>
+      <c r="C18" s="1" t="s">
         <v>49</v>
-      </c>
-      <c r="C18" s="1" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="19" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
+        <v>50</v>
+      </c>
+      <c r="B19" t="s">
         <v>51</v>
       </c>
-      <c r="B19" t="s">
+      <c r="C19" s="1" t="s">
         <v>52</v>
-      </c>
-      <c r="C19" s="1" t="s">
-        <v>53</v>
       </c>
       <c r="D19" t="s">
         <v>8</v>
       </c>
       <c r="E19" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.35">
@@ -1617,10 +1670,10 @@
         <v>20</v>
       </c>
       <c r="B20" t="s">
+        <v>54</v>
+      </c>
+      <c r="C20" s="1" t="s">
         <v>55</v>
-      </c>
-      <c r="C20" s="1" t="s">
-        <v>56</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.35">
@@ -1628,10 +1681,10 @@
         <v>17</v>
       </c>
       <c r="B21" t="s">
+        <v>56</v>
+      </c>
+      <c r="C21" s="1" t="s">
         <v>57</v>
-      </c>
-      <c r="C21" s="1" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="87" x14ac:dyDescent="0.35">
@@ -1639,21 +1692,21 @@
         <v>5</v>
       </c>
       <c r="B22" t="s">
+        <v>58</v>
+      </c>
+      <c r="C22" s="1" t="s">
         <v>59</v>
-      </c>
-      <c r="C22" s="1" t="s">
-        <v>60</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
+        <v>60</v>
+      </c>
+      <c r="B23" t="s">
         <v>61</v>
       </c>
-      <c r="B23" t="s">
+      <c r="C23" s="1" t="s">
         <v>62</v>
-      </c>
-      <c r="C23" s="1" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.35">
@@ -1661,32 +1714,32 @@
         <v>17</v>
       </c>
       <c r="B24" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="C24" s="5" t="s">
         <v>64</v>
-      </c>
-      <c r="C24" s="5" t="s">
-        <v>65</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B25" t="s">
+        <v>65</v>
+      </c>
+      <c r="C25" s="1" t="s">
         <v>66</v>
-      </c>
-      <c r="C25" s="1" t="s">
-        <v>67</v>
       </c>
     </row>
     <row r="26" spans="1:5" ht="58" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
+        <v>67</v>
+      </c>
+      <c r="B26" t="s">
+        <v>50</v>
+      </c>
+      <c r="C26" s="1" t="s">
         <v>68</v>
-      </c>
-      <c r="B26" t="s">
-        <v>51</v>
-      </c>
-      <c r="C26" s="1" t="s">
-        <v>69</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.35">
@@ -1694,10 +1747,10 @@
         <v>17</v>
       </c>
       <c r="B27" t="s">
+        <v>69</v>
+      </c>
+      <c r="C27" s="1" t="s">
         <v>70</v>
-      </c>
-      <c r="C27" s="1" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.35">
@@ -1705,10 +1758,10 @@
         <v>17</v>
       </c>
       <c r="B28" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="C28" s="5" t="s">
         <v>72</v>
-      </c>
-      <c r="C28" s="5" t="s">
-        <v>73</v>
       </c>
     </row>
     <row r="29" spans="1:5" ht="43.5" x14ac:dyDescent="0.35">
@@ -1716,27 +1769,27 @@
         <v>5</v>
       </c>
       <c r="B29" t="s">
+        <v>73</v>
+      </c>
+      <c r="C29" s="1" t="s">
         <v>74</v>
-      </c>
-      <c r="C29" s="1" t="s">
-        <v>75</v>
       </c>
       <c r="D29" t="s">
         <v>15</v>
       </c>
       <c r="E29" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B30" t="s">
+        <v>76</v>
+      </c>
+      <c r="C30" t="s">
         <v>77</v>
-      </c>
-      <c r="C30" t="s">
-        <v>78</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.35">
@@ -1744,10 +1797,10 @@
         <v>17</v>
       </c>
       <c r="B31" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="C31" s="6" t="s">
         <v>79</v>
-      </c>
-      <c r="C31" s="6" t="s">
-        <v>80</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.35">
@@ -1755,10 +1808,10 @@
         <v>20</v>
       </c>
       <c r="B32" t="s">
+        <v>80</v>
+      </c>
+      <c r="C32" s="1" t="s">
         <v>81</v>
-      </c>
-      <c r="C32" s="1" t="s">
-        <v>82</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.35">
@@ -1766,10 +1819,10 @@
         <v>20</v>
       </c>
       <c r="B33" t="s">
+        <v>82</v>
+      </c>
+      <c r="C33" s="1" t="s">
         <v>83</v>
-      </c>
-      <c r="C33" s="1" t="s">
-        <v>84</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.35">
@@ -1777,10 +1830,10 @@
         <v>17</v>
       </c>
       <c r="B34" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="C34" s="5" t="s">
         <v>85</v>
-      </c>
-      <c r="C34" s="5" t="s">
-        <v>86</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.35">
@@ -1788,10 +1841,10 @@
         <v>20</v>
       </c>
       <c r="B35" t="s">
+        <v>86</v>
+      </c>
+      <c r="C35" s="1" t="s">
         <v>87</v>
-      </c>
-      <c r="C35" s="1" t="s">
-        <v>88</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.35">
@@ -1799,21 +1852,21 @@
         <v>17</v>
       </c>
       <c r="B36" t="s">
+        <v>88</v>
+      </c>
+      <c r="C36" s="1" t="s">
         <v>89</v>
-      </c>
-      <c r="C36" s="1" t="s">
-        <v>90</v>
       </c>
     </row>
     <row r="37" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B37" t="s">
+        <v>90</v>
+      </c>
+      <c r="C37" s="1" t="s">
         <v>91</v>
-      </c>
-      <c r="C37" s="1" t="s">
-        <v>92</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.35">
@@ -1821,10 +1874,10 @@
         <v>17</v>
       </c>
       <c r="B38" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="C38" s="1" t="s">
         <v>93</v>
-      </c>
-      <c r="C38" s="1" t="s">
-        <v>94</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.35">
@@ -1832,10 +1885,10 @@
         <v>17</v>
       </c>
       <c r="B39" t="s">
+        <v>94</v>
+      </c>
+      <c r="C39" s="1" t="s">
         <v>95</v>
-      </c>
-      <c r="C39" s="1" t="s">
-        <v>96</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.35">
@@ -1843,10 +1896,10 @@
         <v>17</v>
       </c>
       <c r="B40" t="s">
+        <v>96</v>
+      </c>
+      <c r="C40" s="1" t="s">
         <v>97</v>
-      </c>
-      <c r="C40" s="1" t="s">
-        <v>98</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.35">
@@ -1854,27 +1907,27 @@
         <v>17</v>
       </c>
       <c r="B41" t="s">
+        <v>98</v>
+      </c>
+      <c r="C41" s="1" t="s">
         <v>99</v>
-      </c>
-      <c r="C41" s="1" t="s">
-        <v>100</v>
       </c>
     </row>
     <row r="42" spans="1:5" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B42" t="s">
+        <v>100</v>
+      </c>
+      <c r="C42" s="1" t="s">
         <v>101</v>
-      </c>
-      <c r="C42" s="1" t="s">
-        <v>102</v>
       </c>
       <c r="D42" t="s">
         <v>15</v>
       </c>
       <c r="E42" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.35">
@@ -1882,10 +1935,10 @@
         <v>17</v>
       </c>
       <c r="B43" t="s">
+        <v>103</v>
+      </c>
+      <c r="C43" s="1" t="s">
         <v>104</v>
-      </c>
-      <c r="C43" s="1" t="s">
-        <v>105</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.35">
@@ -1893,10 +1946,10 @@
         <v>17</v>
       </c>
       <c r="B44" t="s">
+        <v>105</v>
+      </c>
+      <c r="C44" s="1" t="s">
         <v>106</v>
-      </c>
-      <c r="C44" s="1" t="s">
-        <v>107</v>
       </c>
     </row>
     <row r="45" spans="1:5" ht="43.5" x14ac:dyDescent="0.35">
@@ -1904,16 +1957,16 @@
         <v>10</v>
       </c>
       <c r="B45" t="s">
+        <v>107</v>
+      </c>
+      <c r="C45" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="C45" s="1" t="s">
+      <c r="D45" t="s">
         <v>109</v>
       </c>
-      <c r="D45" t="s">
+      <c r="E45" t="s">
         <v>110</v>
-      </c>
-      <c r="E45" t="s">
-        <v>111</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.35">
@@ -1921,10 +1974,10 @@
         <v>17</v>
       </c>
       <c r="B46" t="s">
+        <v>111</v>
+      </c>
+      <c r="C46" t="s">
         <v>112</v>
-      </c>
-      <c r="C46" t="s">
-        <v>113</v>
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.35">
@@ -1932,21 +1985,21 @@
         <v>17</v>
       </c>
       <c r="B47" s="5" t="s">
+        <v>113</v>
+      </c>
+      <c r="C47" s="1" t="s">
         <v>114</v>
-      </c>
-      <c r="C47" s="1" t="s">
-        <v>115</v>
       </c>
     </row>
     <row r="48" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
+        <v>115</v>
+      </c>
+      <c r="B48" t="s">
         <v>116</v>
       </c>
-      <c r="B48" t="s">
+      <c r="C48" s="1" t="s">
         <v>117</v>
-      </c>
-      <c r="C48" s="1" t="s">
-        <v>118</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.35">
@@ -1954,21 +2007,21 @@
         <v>17</v>
       </c>
       <c r="B49" t="s">
+        <v>118</v>
+      </c>
+      <c r="C49" s="1" t="s">
         <v>119</v>
-      </c>
-      <c r="C49" s="1" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B50" t="s">
+        <v>120</v>
+      </c>
+      <c r="C50" t="s">
         <v>121</v>
-      </c>
-      <c r="C50" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.35">
@@ -1976,10 +2029,10 @@
         <v>17</v>
       </c>
       <c r="B51" s="5" t="s">
+        <v>122</v>
+      </c>
+      <c r="C51" s="1" t="s">
         <v>123</v>
-      </c>
-      <c r="C51" s="1" t="s">
-        <v>124</v>
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.35">
@@ -1987,10 +2040,10 @@
         <v>17</v>
       </c>
       <c r="B52" t="s">
+        <v>124</v>
+      </c>
+      <c r="C52" s="1" t="s">
         <v>125</v>
-      </c>
-      <c r="C52" s="1" t="s">
-        <v>126</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.35">
@@ -1998,10 +2051,10 @@
         <v>17</v>
       </c>
       <c r="B53" t="s">
+        <v>126</v>
+      </c>
+      <c r="C53" s="1" t="s">
         <v>127</v>
-      </c>
-      <c r="C53" s="1" t="s">
-        <v>128</v>
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.35">
@@ -2009,10 +2062,10 @@
         <v>17</v>
       </c>
       <c r="B54" t="s">
+        <v>128</v>
+      </c>
+      <c r="C54" s="1" t="s">
         <v>129</v>
-      </c>
-      <c r="C54" s="1" t="s">
-        <v>130</v>
       </c>
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.35">
@@ -2020,10 +2073,10 @@
         <v>20</v>
       </c>
       <c r="B55" t="s">
+        <v>130</v>
+      </c>
+      <c r="C55" s="1" t="s">
         <v>131</v>
-      </c>
-      <c r="C55" s="1" t="s">
-        <v>132</v>
       </c>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.35">
@@ -2031,21 +2084,21 @@
         <v>20</v>
       </c>
       <c r="B56" t="s">
+        <v>132</v>
+      </c>
+      <c r="C56" s="1" t="s">
         <v>133</v>
-      </c>
-      <c r="C56" s="1" t="s">
-        <v>134</v>
       </c>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B57" t="s">
+        <v>134</v>
+      </c>
+      <c r="C57" s="1" t="s">
         <v>135</v>
-      </c>
-      <c r="C57" s="1" t="s">
-        <v>136</v>
       </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.35">
@@ -2053,10 +2106,10 @@
         <v>20</v>
       </c>
       <c r="B58" t="s">
+        <v>136</v>
+      </c>
+      <c r="C58" s="1" t="s">
         <v>137</v>
-      </c>
-      <c r="C58" s="1" t="s">
-        <v>138</v>
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.35">
@@ -2064,10 +2117,10 @@
         <v>17</v>
       </c>
       <c r="B59" s="4" t="s">
+        <v>138</v>
+      </c>
+      <c r="C59" s="5" t="s">
         <v>139</v>
-      </c>
-      <c r="C59" s="5" t="s">
-        <v>140</v>
       </c>
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.35">
@@ -2075,21 +2128,21 @@
         <v>17</v>
       </c>
       <c r="B60" s="5" t="s">
+        <v>140</v>
+      </c>
+      <c r="C60" s="1" t="s">
         <v>141</v>
-      </c>
-      <c r="C60" s="1" t="s">
-        <v>142</v>
       </c>
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B61" t="s">
+        <v>142</v>
+      </c>
+      <c r="C61" s="1" t="s">
         <v>143</v>
-      </c>
-      <c r="C61" s="1" t="s">
-        <v>144</v>
       </c>
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.35">
@@ -2097,10 +2150,10 @@
         <v>17</v>
       </c>
       <c r="B62" t="s">
+        <v>144</v>
+      </c>
+      <c r="C62" s="1" t="s">
         <v>145</v>
-      </c>
-      <c r="C62" s="1" t="s">
-        <v>146</v>
       </c>
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.35">
@@ -2108,10 +2161,10 @@
         <v>17</v>
       </c>
       <c r="B63" t="s">
+        <v>146</v>
+      </c>
+      <c r="C63" s="1" t="s">
         <v>147</v>
-      </c>
-      <c r="C63" s="1" t="s">
-        <v>148</v>
       </c>
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.35">
@@ -2119,10 +2172,10 @@
         <v>17</v>
       </c>
       <c r="B64" t="s">
+        <v>148</v>
+      </c>
+      <c r="C64" s="1" t="s">
         <v>149</v>
-      </c>
-      <c r="C64" s="1" t="s">
-        <v>150</v>
       </c>
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.35">
@@ -2130,10 +2183,10 @@
         <v>20</v>
       </c>
       <c r="B65" t="s">
+        <v>150</v>
+      </c>
+      <c r="C65" s="1" t="s">
         <v>151</v>
-      </c>
-      <c r="C65" s="1" t="s">
-        <v>152</v>
       </c>
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.35">
@@ -2141,10 +2194,10 @@
         <v>17</v>
       </c>
       <c r="B66" t="s">
+        <v>152</v>
+      </c>
+      <c r="C66" s="1" t="s">
         <v>153</v>
-      </c>
-      <c r="C66" s="1" t="s">
-        <v>154</v>
       </c>
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.35">
@@ -2152,10 +2205,10 @@
         <v>17</v>
       </c>
       <c r="B67" s="5" t="s">
+        <v>154</v>
+      </c>
+      <c r="C67" s="5" t="s">
         <v>155</v>
-      </c>
-      <c r="C67" s="5" t="s">
-        <v>156</v>
       </c>
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.35">
@@ -2163,21 +2216,21 @@
         <v>17</v>
       </c>
       <c r="B68" t="s">
+        <v>156</v>
+      </c>
+      <c r="C68" s="1" t="s">
         <v>157</v>
-      </c>
-      <c r="C68" s="1" t="s">
-        <v>158</v>
       </c>
     </row>
     <row r="69" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B69" t="s">
+        <v>158</v>
+      </c>
+      <c r="C69" s="1" t="s">
         <v>159</v>
-      </c>
-      <c r="C69" s="1" t="s">
-        <v>160</v>
       </c>
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.35">
@@ -2185,10 +2238,10 @@
         <v>17</v>
       </c>
       <c r="B70" t="s">
+        <v>160</v>
+      </c>
+      <c r="C70" s="1" t="s">
         <v>161</v>
-      </c>
-      <c r="C70" s="1" t="s">
-        <v>162</v>
       </c>
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.35">
@@ -2196,65 +2249,65 @@
         <v>17</v>
       </c>
       <c r="B71" t="s">
+        <v>162</v>
+      </c>
+      <c r="C71" s="1" t="s">
         <v>163</v>
-      </c>
-      <c r="C71" s="1" t="s">
-        <v>164</v>
       </c>
     </row>
     <row r="72" spans="1:5" ht="87" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B72" t="s">
         <v>5</v>
       </c>
       <c r="C72" s="1" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="73" spans="1:5" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
+        <v>166</v>
+      </c>
+      <c r="B73" t="s">
         <v>167</v>
       </c>
-      <c r="B73" t="s">
+      <c r="C73" s="1" t="s">
         <v>168</v>
-      </c>
-      <c r="C73" s="1" t="s">
-        <v>169</v>
       </c>
     </row>
     <row r="74" spans="1:5" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B74" t="s">
+        <v>169</v>
+      </c>
+      <c r="C74" s="4" t="s">
         <v>170</v>
-      </c>
-      <c r="C74" s="4" t="s">
-        <v>171</v>
       </c>
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B75" t="s">
+        <v>171</v>
+      </c>
+      <c r="C75" t="s">
         <v>172</v>
-      </c>
-      <c r="C75" t="s">
-        <v>173</v>
       </c>
     </row>
     <row r="76" spans="1:5" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B76" t="s">
         <v>3</v>
       </c>
       <c r="C76" s="1" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="77" spans="1:5" ht="145" x14ac:dyDescent="0.35">
@@ -2262,10 +2315,10 @@
         <v>10</v>
       </c>
       <c r="B77" s="7" t="s">
+        <v>174</v>
+      </c>
+      <c r="C77" s="10" t="s">
         <v>175</v>
-      </c>
-      <c r="C77" s="10" t="s">
-        <v>176</v>
       </c>
     </row>
     <row r="78" spans="1:5" ht="130.5" x14ac:dyDescent="0.35">
@@ -2273,38 +2326,38 @@
         <v>10</v>
       </c>
       <c r="B78" t="s">
+        <v>176</v>
+      </c>
+      <c r="C78" s="1" t="s">
         <v>177</v>
-      </c>
-      <c r="C78" s="1" t="s">
-        <v>178</v>
       </c>
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B79" t="s">
+        <v>178</v>
+      </c>
+      <c r="C79" s="1" t="s">
         <v>179</v>
-      </c>
-      <c r="C79" s="1" t="s">
-        <v>180</v>
       </c>
       <c r="D79" t="s">
         <v>8</v>
       </c>
       <c r="E79" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="80" spans="1:5" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B80" s="7" t="s">
         <v>10</v>
       </c>
       <c r="C80" s="10" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
     </row>
     <row r="81" spans="1:5" x14ac:dyDescent="0.35">
@@ -2312,32 +2365,32 @@
         <v>17</v>
       </c>
       <c r="B81" s="5" t="s">
+        <v>182</v>
+      </c>
+      <c r="C81" s="5" t="s">
         <v>183</v>
-      </c>
-      <c r="C81" s="5" t="s">
-        <v>184</v>
       </c>
     </row>
     <row r="82" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B82" t="s">
+        <v>184</v>
+      </c>
+      <c r="C82" t="s">
         <v>185</v>
-      </c>
-      <c r="C82" t="s">
-        <v>186</v>
       </c>
     </row>
     <row r="83" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A83" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B83" t="s">
+        <v>186</v>
+      </c>
+      <c r="C83" t="s">
         <v>187</v>
-      </c>
-      <c r="C83" t="s">
-        <v>188</v>
       </c>
     </row>
     <row r="84" spans="1:5" ht="116" x14ac:dyDescent="0.35">
@@ -2345,27 +2398,27 @@
         <v>5</v>
       </c>
       <c r="B84" t="s">
+        <v>188</v>
+      </c>
+      <c r="C84" s="1" t="s">
         <v>189</v>
-      </c>
-      <c r="C84" s="1" t="s">
-        <v>190</v>
       </c>
       <c r="D84" t="s">
         <v>8</v>
       </c>
       <c r="E84" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
     <row r="85" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A85" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B85" t="s">
+        <v>191</v>
+      </c>
+      <c r="C85" s="1" t="s">
         <v>192</v>
-      </c>
-      <c r="C85" s="1" t="s">
-        <v>193</v>
       </c>
     </row>
     <row r="86" spans="1:5" x14ac:dyDescent="0.35">
@@ -2373,10 +2426,10 @@
         <v>17</v>
       </c>
       <c r="B86" s="5" t="s">
+        <v>193</v>
+      </c>
+      <c r="C86" s="1" t="s">
         <v>194</v>
-      </c>
-      <c r="C86" s="1" t="s">
-        <v>195</v>
       </c>
     </row>
     <row r="87" spans="1:5" x14ac:dyDescent="0.35">
@@ -2384,10 +2437,10 @@
         <v>17</v>
       </c>
       <c r="B87" t="s">
+        <v>195</v>
+      </c>
+      <c r="C87" s="1" t="s">
         <v>196</v>
-      </c>
-      <c r="C87" s="1" t="s">
-        <v>197</v>
       </c>
     </row>
     <row r="88" spans="1:5" x14ac:dyDescent="0.35">
@@ -2395,10 +2448,10 @@
         <v>17</v>
       </c>
       <c r="B88" t="s">
+        <v>197</v>
+      </c>
+      <c r="C88" s="1" t="s">
         <v>198</v>
-      </c>
-      <c r="C88" s="1" t="s">
-        <v>199</v>
       </c>
     </row>
     <row r="89" spans="1:5" ht="29" x14ac:dyDescent="0.35">
@@ -2406,10 +2459,10 @@
         <v>17</v>
       </c>
       <c r="B89" t="s">
+        <v>199</v>
+      </c>
+      <c r="C89" s="1" t="s">
         <v>200</v>
-      </c>
-      <c r="C89" s="1" t="s">
-        <v>201</v>
       </c>
     </row>
     <row r="90" spans="1:5" x14ac:dyDescent="0.35">
@@ -2417,10 +2470,10 @@
         <v>17</v>
       </c>
       <c r="B90" t="s">
+        <v>201</v>
+      </c>
+      <c r="C90" s="1" t="s">
         <v>202</v>
-      </c>
-      <c r="C90" s="1" t="s">
-        <v>203</v>
       </c>
     </row>
     <row r="91" spans="1:5" x14ac:dyDescent="0.35">
@@ -2428,10 +2481,10 @@
         <v>17</v>
       </c>
       <c r="B91" t="s">
+        <v>203</v>
+      </c>
+      <c r="C91" s="1" t="s">
         <v>204</v>
-      </c>
-      <c r="C91" s="1" t="s">
-        <v>205</v>
       </c>
     </row>
     <row r="92" spans="1:5" x14ac:dyDescent="0.35">
@@ -2439,21 +2492,21 @@
         <v>17</v>
       </c>
       <c r="B92" s="5" t="s">
+        <v>205</v>
+      </c>
+      <c r="C92" s="1" t="s">
         <v>206</v>
-      </c>
-      <c r="C92" s="1" t="s">
-        <v>207</v>
       </c>
     </row>
     <row r="93" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A93" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B93" t="s">
+        <v>207</v>
+      </c>
+      <c r="C93" t="s">
         <v>208</v>
-      </c>
-      <c r="C93" t="s">
-        <v>209</v>
       </c>
     </row>
     <row r="94" spans="1:5" x14ac:dyDescent="0.35">
@@ -2461,10 +2514,10 @@
         <v>20</v>
       </c>
       <c r="B94" t="s">
+        <v>209</v>
+      </c>
+      <c r="C94" s="1" t="s">
         <v>210</v>
-      </c>
-      <c r="C94" s="1" t="s">
-        <v>211</v>
       </c>
     </row>
     <row r="95" spans="1:5" x14ac:dyDescent="0.35">
@@ -2472,21 +2525,21 @@
         <v>17</v>
       </c>
       <c r="B95" s="5" t="s">
+        <v>211</v>
+      </c>
+      <c r="C95" s="1" t="s">
         <v>212</v>
-      </c>
-      <c r="C95" s="1" t="s">
-        <v>213</v>
       </c>
     </row>
     <row r="96" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A96" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B96" t="s">
+        <v>213</v>
+      </c>
+      <c r="C96" s="1" t="s">
         <v>214</v>
-      </c>
-      <c r="C96" s="1" t="s">
-        <v>215</v>
       </c>
     </row>
     <row r="97" spans="1:5" ht="29" x14ac:dyDescent="0.35">
@@ -2494,44 +2547,44 @@
         <v>39</v>
       </c>
       <c r="B97" t="s">
+        <v>215</v>
+      </c>
+      <c r="C97" s="9" t="s">
         <v>216</v>
-      </c>
-      <c r="C97" s="9" t="s">
-        <v>217</v>
       </c>
       <c r="D97" t="s">
         <v>15</v>
       </c>
       <c r="E97" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="98" spans="1:5" ht="58" x14ac:dyDescent="0.35">
       <c r="A98" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B98" t="s">
+        <v>218</v>
+      </c>
+      <c r="C98" s="1" t="s">
         <v>219</v>
-      </c>
-      <c r="C98" s="1" t="s">
-        <v>220</v>
       </c>
     </row>
     <row r="99" spans="1:5" ht="130.5" x14ac:dyDescent="0.35">
       <c r="A99" t="s">
+        <v>220</v>
+      </c>
+      <c r="B99" t="s">
         <v>221</v>
       </c>
-      <c r="B99" t="s">
+      <c r="C99" s="1" t="s">
         <v>222</v>
-      </c>
-      <c r="C99" s="1" t="s">
-        <v>223</v>
       </c>
       <c r="D99" t="s">
         <v>15</v>
       </c>
       <c r="E99" s="11" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="100" spans="1:5" x14ac:dyDescent="0.35">
@@ -2539,10 +2592,10 @@
         <v>17</v>
       </c>
       <c r="B100" t="s">
+        <v>224</v>
+      </c>
+      <c r="C100" s="8" t="s">
         <v>225</v>
-      </c>
-      <c r="C100" s="8" t="s">
-        <v>226</v>
       </c>
     </row>
     <row r="101" spans="1:5" x14ac:dyDescent="0.35">
@@ -2550,10 +2603,10 @@
         <v>17</v>
       </c>
       <c r="B101" t="s">
+        <v>226</v>
+      </c>
+      <c r="C101" s="1" t="s">
         <v>227</v>
-      </c>
-      <c r="C101" s="1" t="s">
-        <v>228</v>
       </c>
     </row>
     <row r="102" spans="1:5" x14ac:dyDescent="0.35">
@@ -2561,10 +2614,10 @@
         <v>17</v>
       </c>
       <c r="B102" t="s">
+        <v>228</v>
+      </c>
+      <c r="C102" s="1" t="s">
         <v>229</v>
-      </c>
-      <c r="C102" s="1" t="s">
-        <v>230</v>
       </c>
     </row>
     <row r="103" spans="1:5" x14ac:dyDescent="0.35">
@@ -2572,10 +2625,10 @@
         <v>20</v>
       </c>
       <c r="B103" t="s">
+        <v>230</v>
+      </c>
+      <c r="C103" s="1" t="s">
         <v>231</v>
-      </c>
-      <c r="C103" s="1" t="s">
-        <v>232</v>
       </c>
     </row>
     <row r="104" spans="1:5" x14ac:dyDescent="0.35">
@@ -2583,10 +2636,10 @@
         <v>17</v>
       </c>
       <c r="B104" t="s">
+        <v>232</v>
+      </c>
+      <c r="C104" s="1" t="s">
         <v>233</v>
-      </c>
-      <c r="C104" s="1" t="s">
-        <v>234</v>
       </c>
     </row>
     <row r="105" spans="1:5" x14ac:dyDescent="0.35">
@@ -2594,27 +2647,27 @@
         <v>17</v>
       </c>
       <c r="B105" t="s">
+        <v>234</v>
+      </c>
+      <c r="C105" s="1" t="s">
         <v>235</v>
-      </c>
-      <c r="C105" s="1" t="s">
-        <v>236</v>
       </c>
     </row>
     <row r="106" spans="1:5" ht="58" x14ac:dyDescent="0.35">
       <c r="A106" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B106" t="s">
+        <v>236</v>
+      </c>
+      <c r="C106" s="1" t="s">
         <v>237</v>
-      </c>
-      <c r="C106" s="1" t="s">
-        <v>238</v>
       </c>
       <c r="D106" t="s">
         <v>15</v>
       </c>
       <c r="E106" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="107" spans="1:5" ht="130.5" x14ac:dyDescent="0.35">
@@ -2622,16 +2675,16 @@
         <v>10</v>
       </c>
       <c r="B107" t="s">
+        <v>239</v>
+      </c>
+      <c r="C107" s="1" t="s">
         <v>240</v>
-      </c>
-      <c r="C107" s="1" t="s">
-        <v>241</v>
       </c>
       <c r="D107" t="s">
         <v>15</v>
       </c>
       <c r="E107" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="108" spans="1:5" x14ac:dyDescent="0.35">
@@ -2639,10 +2692,10 @@
         <v>17</v>
       </c>
       <c r="B108" t="s">
+        <v>242</v>
+      </c>
+      <c r="C108" s="1" t="s">
         <v>243</v>
-      </c>
-      <c r="C108" s="1" t="s">
-        <v>244</v>
       </c>
     </row>
     <row r="109" spans="1:5" x14ac:dyDescent="0.35">
@@ -2650,10 +2703,10 @@
         <v>17</v>
       </c>
       <c r="B109" t="s">
+        <v>244</v>
+      </c>
+      <c r="C109" s="1" t="s">
         <v>245</v>
-      </c>
-      <c r="C109" s="1" t="s">
-        <v>246</v>
       </c>
     </row>
     <row r="110" spans="1:5" x14ac:dyDescent="0.35">
@@ -2661,10 +2714,10 @@
         <v>17</v>
       </c>
       <c r="B110" t="s">
+        <v>246</v>
+      </c>
+      <c r="C110" s="1" t="s">
         <v>247</v>
-      </c>
-      <c r="C110" s="1" t="s">
-        <v>248</v>
       </c>
     </row>
     <row r="111" spans="1:5" x14ac:dyDescent="0.35">
@@ -2672,10 +2725,10 @@
         <v>17</v>
       </c>
       <c r="B111" t="s">
+        <v>248</v>
+      </c>
+      <c r="C111" s="1" t="s">
         <v>249</v>
-      </c>
-      <c r="C111" s="1" t="s">
-        <v>250</v>
       </c>
     </row>
     <row r="112" spans="1:5" x14ac:dyDescent="0.35">
@@ -2683,10 +2736,10 @@
         <v>17</v>
       </c>
       <c r="B112" t="s">
+        <v>250</v>
+      </c>
+      <c r="C112" s="1" t="s">
         <v>251</v>
-      </c>
-      <c r="C112" s="1" t="s">
-        <v>252</v>
       </c>
     </row>
     <row r="113" spans="1:3" x14ac:dyDescent="0.35">
@@ -2694,10 +2747,10 @@
         <v>17</v>
       </c>
       <c r="B113" t="s">
+        <v>252</v>
+      </c>
+      <c r="C113" s="1" t="s">
         <v>253</v>
-      </c>
-      <c r="C113" s="1" t="s">
-        <v>254</v>
       </c>
     </row>
     <row r="114" spans="1:3" ht="29" x14ac:dyDescent="0.35">
@@ -2705,10 +2758,10 @@
         <v>17</v>
       </c>
       <c r="B114" t="s">
+        <v>254</v>
+      </c>
+      <c r="C114" s="1" t="s">
         <v>255</v>
-      </c>
-      <c r="C114" s="1" t="s">
-        <v>256</v>
       </c>
     </row>
     <row r="115" spans="1:3" x14ac:dyDescent="0.35">
@@ -2716,10 +2769,10 @@
         <v>17</v>
       </c>
       <c r="B115" t="s">
+        <v>256</v>
+      </c>
+      <c r="C115" s="1" t="s">
         <v>257</v>
-      </c>
-      <c r="C115" s="1" t="s">
-        <v>258</v>
       </c>
     </row>
     <row r="116" spans="1:3" x14ac:dyDescent="0.35">
@@ -2727,10 +2780,10 @@
         <v>17</v>
       </c>
       <c r="B116" t="s">
+        <v>258</v>
+      </c>
+      <c r="C116" s="1" t="s">
         <v>259</v>
-      </c>
-      <c r="C116" s="1" t="s">
-        <v>260</v>
       </c>
     </row>
     <row r="117" spans="1:3" x14ac:dyDescent="0.35">
@@ -2738,10 +2791,10 @@
         <v>17</v>
       </c>
       <c r="B117" t="s">
+        <v>260</v>
+      </c>
+      <c r="C117" s="1" t="s">
         <v>261</v>
-      </c>
-      <c r="C117" s="1" t="s">
-        <v>262</v>
       </c>
     </row>
     <row r="118" spans="1:3" x14ac:dyDescent="0.35">
@@ -2749,10 +2802,10 @@
         <v>17</v>
       </c>
       <c r="B118" t="s">
+        <v>262</v>
+      </c>
+      <c r="C118" s="1" t="s">
         <v>263</v>
-      </c>
-      <c r="C118" s="1" t="s">
-        <v>264</v>
       </c>
     </row>
     <row r="119" spans="1:3" x14ac:dyDescent="0.35">
@@ -2760,10 +2813,10 @@
         <v>17</v>
       </c>
       <c r="B119" t="s">
+        <v>264</v>
+      </c>
+      <c r="C119" s="1" t="s">
         <v>265</v>
-      </c>
-      <c r="C119" s="1" t="s">
-        <v>266</v>
       </c>
     </row>
     <row r="120" spans="1:3" x14ac:dyDescent="0.35">
@@ -2771,10 +2824,10 @@
         <v>17</v>
       </c>
       <c r="B120" t="s">
+        <v>266</v>
+      </c>
+      <c r="C120" s="1" t="s">
         <v>267</v>
-      </c>
-      <c r="C120" s="1" t="s">
-        <v>268</v>
       </c>
     </row>
     <row r="121" spans="1:3" x14ac:dyDescent="0.35">
@@ -2782,10 +2835,10 @@
         <v>17</v>
       </c>
       <c r="B121" t="s">
+        <v>268</v>
+      </c>
+      <c r="C121" s="1" t="s">
         <v>269</v>
-      </c>
-      <c r="C121" s="1" t="s">
-        <v>270</v>
       </c>
     </row>
     <row r="122" spans="1:3" x14ac:dyDescent="0.35">
@@ -2793,10 +2846,10 @@
         <v>17</v>
       </c>
       <c r="B122" s="12" t="s">
+        <v>270</v>
+      </c>
+      <c r="C122" s="12" t="s">
         <v>271</v>
-      </c>
-      <c r="C122" s="12" t="s">
-        <v>272</v>
       </c>
     </row>
     <row r="123" spans="1:3" x14ac:dyDescent="0.35">
@@ -2804,10 +2857,10 @@
         <v>17</v>
       </c>
       <c r="B123" s="13" t="s">
+        <v>272</v>
+      </c>
+      <c r="C123" s="13" t="s">
         <v>273</v>
-      </c>
-      <c r="C123" s="13" t="s">
-        <v>274</v>
       </c>
     </row>
     <row r="124" spans="1:3" x14ac:dyDescent="0.35">
@@ -2815,10 +2868,10 @@
         <v>17</v>
       </c>
       <c r="B124" t="s">
+        <v>274</v>
+      </c>
+      <c r="C124" t="s">
         <v>275</v>
-      </c>
-      <c r="C124" t="s">
-        <v>276</v>
       </c>
     </row>
     <row r="125" spans="1:3" x14ac:dyDescent="0.35">
@@ -2826,10 +2879,10 @@
         <v>17</v>
       </c>
       <c r="B125" t="s">
+        <v>276</v>
+      </c>
+      <c r="C125" s="1" t="s">
         <v>277</v>
-      </c>
-      <c r="C125" s="1" t="s">
-        <v>278</v>
       </c>
     </row>
     <row r="126" spans="1:3" x14ac:dyDescent="0.35">
@@ -2837,10 +2890,10 @@
         <v>17</v>
       </c>
       <c r="B126" t="s">
+        <v>278</v>
+      </c>
+      <c r="C126" s="1" t="s">
         <v>279</v>
-      </c>
-      <c r="C126" s="1" t="s">
-        <v>280</v>
       </c>
     </row>
     <row r="127" spans="1:3" x14ac:dyDescent="0.35">
@@ -2848,10 +2901,10 @@
         <v>17</v>
       </c>
       <c r="B127" t="s">
+        <v>280</v>
+      </c>
+      <c r="C127" s="1" t="s">
         <v>281</v>
-      </c>
-      <c r="C127" s="1" t="s">
-        <v>282</v>
       </c>
     </row>
     <row r="128" spans="1:3" x14ac:dyDescent="0.35">
@@ -2859,10 +2912,10 @@
         <v>17</v>
       </c>
       <c r="B128" t="s">
+        <v>282</v>
+      </c>
+      <c r="C128" s="1" t="s">
         <v>283</v>
-      </c>
-      <c r="C128" s="1" t="s">
-        <v>284</v>
       </c>
     </row>
     <row r="129" spans="1:3" x14ac:dyDescent="0.35">
@@ -2870,10 +2923,10 @@
         <v>17</v>
       </c>
       <c r="B129" t="s">
+        <v>284</v>
+      </c>
+      <c r="C129" s="1" t="s">
         <v>285</v>
-      </c>
-      <c r="C129" s="1" t="s">
-        <v>286</v>
       </c>
     </row>
     <row r="130" spans="1:3" x14ac:dyDescent="0.35">
@@ -2881,10 +2934,65 @@
         <v>17</v>
       </c>
       <c r="B130" t="s">
+        <v>286</v>
+      </c>
+      <c r="C130" s="14" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="131" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A131" t="s">
+        <v>17</v>
+      </c>
+      <c r="B131" t="s">
         <v>287</v>
       </c>
-      <c r="C130" s="14" t="s">
+      <c r="C131" s="15" t="s">
         <v>288</v>
+      </c>
+    </row>
+    <row r="132" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A132" t="s">
+        <v>17</v>
+      </c>
+      <c r="B132" t="s">
+        <v>289</v>
+      </c>
+      <c r="C132" s="15" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="133" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A133" t="s">
+        <v>17</v>
+      </c>
+      <c r="B133" t="s">
+        <v>291</v>
+      </c>
+      <c r="C133" s="1" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="134" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A134" t="s">
+        <v>17</v>
+      </c>
+      <c r="B134" t="s">
+        <v>293</v>
+      </c>
+      <c r="C134" s="1" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="135" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A135" t="s">
+        <v>17</v>
+      </c>
+      <c r="B135" t="s">
+        <v>296</v>
+      </c>
+      <c r="C135" s="1" t="s">
+        <v>295</v>
       </c>
     </row>
   </sheetData>
@@ -3149,15 +3257,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="00850a8a-55a0-4f29-bb56-d3de9b9bc75c">
@@ -3166,6 +3265,15 @@
     <TaxCatchAll xmlns="33e70369-3675-4c3b-99e1-030eb9633bdf" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3188,26 +3296,26 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{13521947-7B63-4043-9A52-D2F3EDCA31C1}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="33e70369-3675-4c3b-99e1-030eb9633bdf"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="00850a8a-55a0-4f29-bb56-d3de9b9bc75c"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F7554B1E-EA5B-4036-8BEB-CEB54DFFA990}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{13521947-7B63-4043-9A52-D2F3EDCA31C1}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="33e70369-3675-4c3b-99e1-030eb9633bdf"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="00850a8a-55a0-4f29-bb56-d3de9b9bc75c"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>